<commit_message>
new sensor update: changed processing and normalization functions
</commit_message>
<xml_diff>
--- a/Codigos/Windows/Registro Pacientes.xlsx
+++ b/Codigos/Windows/Registro Pacientes.xlsx
@@ -1,72 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zakie Assad\Proyecto Final\Git\MoAna\Codigos\Windows\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D045A120-B56E-433D-B6A9-8B11E4237C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>fecha</t>
-  </si>
-  <si>
-    <t>hora</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>nombre</t>
-  </si>
-  <si>
-    <t>apellido</t>
-  </si>
-  <si>
-    <t>Archivo Informe</t>
-  </si>
-  <si>
-    <t>Archivo Datos</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -84,23 +55,84 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -400,41 +432,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="4" max="5" width="20.85546875" customWidth="1"/>
-    <col min="6" max="6" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col width="14.140625" customWidth="1" min="1" max="1"/>
+    <col width="18.85546875" customWidth="1" min="2" max="2"/>
+    <col width="20.85546875" customWidth="1" min="4" max="5"/>
+    <col width="35.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="33.140625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="15" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1"/>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>hora</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>apellido</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo Informe</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo Datos</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>45141</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.616785775462963</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8654323456</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LUCILA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CAPURRO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Informe 8654323456 2023-08-03 14.48.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Datos 8654323456 2023-08-03 14.48.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>45141</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.6248957550925927</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FGH</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Informe RTY 2023-08-03 14.59.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Datos RTY 2023-08-03 14.59.csv</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
cambio de fs a 25 y 500 + norma alarmas + estetica interfaz
</commit_message>
<xml_diff>
--- a/Codigos/Windows/Registro Pacientes.xlsx
+++ b/Codigos/Windows/Registro Pacientes.xlsx
@@ -1,72 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zakie Assad\Proyecto Final\Git\MoAna\Codigos\Windows\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9105BE4-554B-4935-A1C2-BE5C747DCF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>fecha</t>
-  </si>
-  <si>
-    <t>hora</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>nombre</t>
-  </si>
-  <si>
-    <t>apellido</t>
-  </si>
-  <si>
-    <t>Archivo Informe</t>
-  </si>
-  <si>
-    <t>Archivo Datos</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -84,23 +55,84 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -400,41 +432,191 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="4" max="5" width="20.85546875" customWidth="1"/>
-    <col min="6" max="6" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
+    <col width="14.140625" customWidth="1" min="1" max="1"/>
+    <col width="18.85546875" customWidth="1" min="2" max="2"/>
+    <col width="20.85546875" customWidth="1" min="4" max="5"/>
+    <col width="35.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="33.140625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="15" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1"/>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>hora</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>apellido</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo Informe</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo Datos</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>45187</v>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.5678287847222222</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>fs</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fs</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>fs</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Informe fs 2023-09-18 13.37.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Datos fs 2023-09-18 13.37.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>45194</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.7824137962962963</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>probando fs 25!!!</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>probando fs 25!!!</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>probando fs 25!!!</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Informe probando fs 25!!! 2023-09-25 18.46.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Datos probando fs 25!!! 2023-09-25 18.46.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>45198</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.7515351967592593</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>,</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Informe , 2023-09-29 18.02.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Datos , 2023-09-29 18.02.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>45198</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.752288188287037</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>asd</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>zakie</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>assad</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Informe asd 2023-09-29 18.03.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Datos asd 2023-09-29 18.03.csv</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
cambio sonidos alarmas + guardado de alarmas
</commit_message>
<xml_diff>
--- a/Codigos/Windows/Registro Pacientes.xlsx
+++ b/Codigos/Windows/Registro Pacientes.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="14.140625" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
         <v>45198</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.752288188287037</v>
+        <v>0.7522881828703704</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -615,6 +615,237 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>Datos asd 2023-09-29 18.03.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.4313986574074073</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Informe sdf 2023-10-01 10.21.pdf</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Datos sdf 2023-10-01 10.21.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.4366816782407407</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>kn</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Informe k 2023-10-01 10.28.pdf</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Datos k 2023-10-01 10.28.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.4509079050925926</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Informe sdf 2023-10-01 10.49.pdf</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Datos sdf 2023-10-01 10.49.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.4566550810185185</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>zakie</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>zakie</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>zakie</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Informe zakie 2023-10-01 10.57.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Datos zakie 2023-10-01 10.57.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.4666727546296296</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>zak</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>zaki</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>zakio</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Informe zak 2023-10-01 11.12.pdf</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Datos zak 2023-10-01 11.12.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.4719139583333333</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>df</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>sdvsdf</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Informe df 2023-10-01 11.19.pdf</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Datos df 2023-10-01 11.19.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.4766553821180555</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>sdf</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>asd</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>df</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Informe sdf 2023-10-01 11.26.pdf</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Datos sdf 2023-10-01 11.26.csv</t>
         </is>
       </c>
     </row>

</xml_diff>